<commit_message>
fix: the example's AE block counts treatment-emergent events
Its <System Organ Class> / <Preferred Term> rows carried no filter, so
the block counted every adverse event under a table headed
"Treatment-Emergent Adverse Events" -- 12 Placebo subjects with a nervous
system event where 8 had a treatment-emergent one.

Nothing propagates the "Subjects with any TEAE" row's filter down a
block, so each token row now carries WHERE ADAE.TRTEMFL='Y' itself. The
bundle test checks the numbers against the raw dataset rather than
against the pipeline that produced them.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/inst/extdata/example_cdsc_alz_201/annotated_shell.xlsx
+++ b/inst/extdata/example_cdsc_alz_201/annotated_shell.xlsx
@@ -1230,7 +1230,7 @@
               <color rgb="FFC00000"/>
             </rPr>
             <t xml:space="preserve">
-[ADAE.AESOC]</t>
+[ADAE.AESOC WHERE ADAE.TRTEMFL='Y']</t>
           </r>
         </is>
       </c>
@@ -1267,7 +1267,7 @@
               <color rgb="FFC00000"/>
             </rPr>
             <t xml:space="preserve">
-[ADAE.AEDECOD]</t>
+[ADAE.AEDECOD WHERE ADAE.TRTEMFL='Y']</t>
           </r>
         </is>
       </c>

</xml_diff>

<commit_message>
feat: the bundled shells name the ADSL treatment variable
The reference shell should show the form the parser recommends. Every
table's column axis now names ADSL.TRT01A, whatever domain its data comes
from, so the bundle parses without a column-axis finding.

The numbers are unchanged -- ADAE and ADEX carry TRT01A with ADSL's
values, which is why that case was an INFO rather than a WARN. ADCM does
not carry it, so its listing still reads ADCM.TRTA: a listing has no
denominator to split, and the same edit there would leave every cell
pending.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/inst/extdata/example_cdsc_alz_201/annotated_shell.xlsx
+++ b/inst/extdata/example_cdsc_alz_201/annotated_shell.xlsx
@@ -897,7 +897,7 @@
               <color rgb="FFC00000"/>
             </rPr>
             <t xml:space="preserve">
-[columns -&gt; ADAE.TRT01A; source ADAE]</t>
+[columns -&gt; ADSL.TRT01A; source ADAE]</t>
           </r>
         </is>
       </c>
@@ -1156,7 +1156,7 @@
               <color rgb="FFC00000"/>
             </rPr>
             <t xml:space="preserve">
-[columns -&gt; ADAE.TRT01A; source ADAE]</t>
+[columns -&gt; ADSL.TRT01A; source ADAE]</t>
           </r>
         </is>
       </c>
@@ -1364,7 +1364,7 @@
               <color rgb="FFC00000"/>
             </rPr>
             <t xml:space="preserve">
-[columns -&gt; ADEX.TRT01A; source ADEX]</t>
+[columns -&gt; ADSL.TRT01A; source ADEX]</t>
           </r>
         </is>
       </c>

</xml_diff>